<commit_message>
Optimize framework: Add headless capability, resolve ESM imports, and enable 4-worker parallel xdist pipelines
</commit_message>
<xml_diff>
--- a/UIBank/TestData/RegistrationData.xlsx
+++ b/UIBank/TestData/RegistrationData.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\NG5347\PycharmProjects\SizweSelfLearningPOE-Python\UIBank\TestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{91B9FA1F-14D8-445A-A3BF-DBCF4D21BD89}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9816ADA5-1F96-44EC-BBCF-7E6076A96444}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-1515" windowWidth="29040" windowHeight="15720" xr2:uid="{A6B4279B-6C98-4A1E-A258-309E602C7628}"/>
   </bookViews>
@@ -104,9 +104,6 @@
     <t>Full-Time</t>
   </si>
   <si>
-    <t>01/15/1988</t>
-  </si>
-  <si>
     <t>Married</t>
   </si>
   <si>
@@ -134,9 +131,6 @@
     <t>Part-Time</t>
   </si>
   <si>
-    <t>03/22/1992</t>
-  </si>
-  <si>
     <t>Single</t>
   </si>
   <si>
@@ -155,9 +149,6 @@
     <t>C</t>
   </si>
   <si>
-    <t>07/08/1985</t>
-  </si>
-  <si>
     <t>michaelwilliams03</t>
   </si>
   <si>
@@ -179,9 +170,6 @@
     <t>Self-Employed</t>
   </si>
   <si>
-    <t>11/30/1990</t>
-  </si>
-  <si>
     <t>emilybrown04</t>
   </si>
   <si>
@@ -197,9 +185,6 @@
     <t>E</t>
   </si>
   <si>
-    <t>05/12/1987</t>
-  </si>
-  <si>
     <t>davidjones05</t>
   </si>
   <si>
@@ -218,9 +203,6 @@
     <t>Student</t>
   </si>
   <si>
-    <t>04/18/1998</t>
-  </si>
-  <si>
     <t>jessicagarcia06</t>
   </si>
   <si>
@@ -236,9 +218,6 @@
     <t>G</t>
   </si>
   <si>
-    <t>09/03/1984</t>
-  </si>
-  <si>
     <t>matthewmiller07</t>
   </si>
   <si>
@@ -254,9 +233,6 @@
     <t>H</t>
   </si>
   <si>
-    <t>12/21/1993</t>
-  </si>
-  <si>
     <t>ashleydavis08</t>
   </si>
   <si>
@@ -272,9 +248,6 @@
     <t>I</t>
   </si>
   <si>
-    <t>08/10/1986</t>
-  </si>
-  <si>
     <t>christophermartinez09</t>
   </si>
   <si>
@@ -290,9 +263,6 @@
     <t>J</t>
   </si>
   <si>
-    <t>02/27/1989</t>
-  </si>
-  <si>
     <t>amandahernandez10</t>
   </si>
   <si>
@@ -308,9 +278,6 @@
     <t>K</t>
   </si>
   <si>
-    <t>06/14/1983</t>
-  </si>
-  <si>
     <t>Divorced</t>
   </si>
   <si>
@@ -329,9 +296,6 @@
     <t>L</t>
   </si>
   <si>
-    <t>09/09/1991</t>
-  </si>
-  <si>
     <t>jennifergonzalez12</t>
   </si>
   <si>
@@ -347,9 +311,6 @@
     <t>M</t>
   </si>
   <si>
-    <t>01/07/1982</t>
-  </si>
-  <si>
     <t>joshuawilson13</t>
   </si>
   <si>
@@ -365,9 +326,6 @@
     <t>N</t>
   </si>
   <si>
-    <t>10/25/1988</t>
-  </si>
-  <si>
     <t>melissaanderson14</t>
   </si>
   <si>
@@ -386,9 +344,6 @@
     <t>Dr</t>
   </si>
   <si>
-    <t>03/17/1980</t>
-  </si>
-  <si>
     <t>andrewthomas15</t>
   </si>
   <si>
@@ -404,9 +359,6 @@
     <t>P</t>
   </si>
   <si>
-    <t>07/11/1999</t>
-  </si>
-  <si>
     <t>nicoletaylor16</t>
   </si>
   <si>
@@ -422,9 +374,6 @@
     <t>Q</t>
   </si>
   <si>
-    <t>11/19/1987</t>
-  </si>
-  <si>
     <t>ryanmoore17</t>
   </si>
   <si>
@@ -440,9 +389,6 @@
     <t>R</t>
   </si>
   <si>
-    <t>05/22/1990</t>
-  </si>
-  <si>
     <t>samanthajackson18</t>
   </si>
   <si>
@@ -458,9 +404,6 @@
     <t>S</t>
   </si>
   <si>
-    <t>04/16/1985</t>
-  </si>
-  <si>
     <t>brandonmartin19</t>
   </si>
   <si>
@@ -476,9 +419,6 @@
     <t>T</t>
   </si>
   <si>
-    <t>08/29/1994</t>
-  </si>
-  <si>
     <t>laurenlee20</t>
   </si>
   <si>
@@ -494,9 +434,6 @@
     <t>U</t>
   </si>
   <si>
-    <t>12/13/1986</t>
-  </si>
-  <si>
     <t>justinperez21</t>
   </si>
   <si>
@@ -512,9 +449,6 @@
     <t>V</t>
   </si>
   <si>
-    <t>06/20/1989</t>
-  </si>
-  <si>
     <t>meganthompson22</t>
   </si>
   <si>
@@ -530,9 +464,6 @@
     <t>W</t>
   </si>
   <si>
-    <t>09/02/1992</t>
-  </si>
-  <si>
     <t>kevinwhite23</t>
   </si>
   <si>
@@ -548,9 +479,6 @@
     <t>X</t>
   </si>
   <si>
-    <t>02/08/1984</t>
-  </si>
-  <si>
     <t>rachelharris24</t>
   </si>
   <si>
@@ -566,9 +494,6 @@
     <t>Y</t>
   </si>
   <si>
-    <t>04/04/1988</t>
-  </si>
-  <si>
     <t>tylersanchez25</t>
   </si>
   <si>
@@ -584,9 +509,6 @@
     <t>Z</t>
   </si>
   <si>
-    <t>10/10/1999</t>
-  </si>
-  <si>
     <t>kaylaclark26</t>
   </si>
   <si>
@@ -599,9 +521,6 @@
     <t>Ramirez</t>
   </si>
   <si>
-    <t>07/27/1983</t>
-  </si>
-  <si>
     <t>nicholasramirez27</t>
   </si>
   <si>
@@ -614,9 +533,6 @@
     <t>Lewis</t>
   </si>
   <si>
-    <t>01/18/1987</t>
-  </si>
-  <si>
     <t>olivialewis28</t>
   </si>
   <si>
@@ -629,9 +545,6 @@
     <t>Robinson</t>
   </si>
   <si>
-    <t>05/31/1981</t>
-  </si>
-  <si>
     <t>jonathanrobinson29</t>
   </si>
   <si>
@@ -644,9 +557,6 @@
     <t>Walker</t>
   </si>
   <si>
-    <t>09/14/1995</t>
-  </si>
-  <si>
     <t>hannahwalker30</t>
   </si>
   <si>
@@ -659,9 +569,6 @@
     <t>Young</t>
   </si>
   <si>
-    <t>03/09/1982</t>
-  </si>
-  <si>
     <t>patrickyoung31</t>
   </si>
   <si>
@@ -674,9 +581,6 @@
     <t>Allen</t>
   </si>
   <si>
-    <t>06/06/1988</t>
-  </si>
-  <si>
     <t>abigailallen32</t>
   </si>
   <si>
@@ -689,9 +593,6 @@
     <t>King</t>
   </si>
   <si>
-    <t>11/22/1985</t>
-  </si>
-  <si>
     <t>ethanking33</t>
   </si>
   <si>
@@ -704,9 +605,6 @@
     <t>Wright</t>
   </si>
   <si>
-    <t>08/30/1998</t>
-  </si>
-  <si>
     <t>gracewright34</t>
   </si>
   <si>
@@ -719,9 +617,6 @@
     <t>Scott</t>
   </si>
   <si>
-    <t>04/12/1984</t>
-  </si>
-  <si>
     <t>benjaminscott35</t>
   </si>
   <si>
@@ -734,9 +629,6 @@
     <t>Torres</t>
   </si>
   <si>
-    <t>12/01/1991</t>
-  </si>
-  <si>
     <t>victoriatorres36</t>
   </si>
   <si>
@@ -749,9 +641,6 @@
     <t>Nguyen</t>
   </si>
   <si>
-    <t>07/16/1986</t>
-  </si>
-  <si>
     <t>nathannguyen37</t>
   </si>
   <si>
@@ -764,9 +653,6 @@
     <t>Hill</t>
   </si>
   <si>
-    <t>01/25/1993</t>
-  </si>
-  <si>
     <t>chloehill38</t>
   </si>
   <si>
@@ -779,9 +665,6 @@
     <t>Flores</t>
   </si>
   <si>
-    <t>10/05/1987</t>
-  </si>
-  <si>
     <t>christianflores39</t>
   </si>
   <si>
@@ -794,9 +677,6 @@
     <t>Green</t>
   </si>
   <si>
-    <t>03/11/1990</t>
-  </si>
-  <si>
     <t>nataliegreen40</t>
   </si>
   <si>
@@ -809,9 +689,6 @@
     <t>Adams</t>
   </si>
   <si>
-    <t>06/27/1994</t>
-  </si>
-  <si>
     <t>aaronadams41</t>
   </si>
   <si>
@@ -824,9 +701,6 @@
     <t>Nelson</t>
   </si>
   <si>
-    <t>09/17/2000</t>
-  </si>
-  <si>
     <t>zoenelson42</t>
   </si>
   <si>
@@ -839,9 +713,6 @@
     <t>Baker</t>
   </si>
   <si>
-    <t>02/02/1985</t>
-  </si>
-  <si>
     <t>jasonbaker43</t>
   </si>
   <si>
@@ -854,9 +725,6 @@
     <t>Hall</t>
   </si>
   <si>
-    <t>11/13/1988</t>
-  </si>
-  <si>
     <t>faithhall44</t>
   </si>
   <si>
@@ -869,9 +737,6 @@
     <t>Campbell</t>
   </si>
   <si>
-    <t>05/21/1983</t>
-  </si>
-  <si>
     <t>kylecampbell45</t>
   </si>
   <si>
@@ -884,9 +749,6 @@
     <t>Mitchell</t>
   </si>
   <si>
-    <t>08/08/1992</t>
-  </si>
-  <si>
     <t>brookemitchell46</t>
   </si>
   <si>
@@ -899,9 +761,6 @@
     <t>Carter</t>
   </si>
   <si>
-    <t>01/29/1986</t>
-  </si>
-  <si>
     <t>seancarter47</t>
   </si>
   <si>
@@ -914,9 +773,6 @@
     <t>Roberts</t>
   </si>
   <si>
-    <t>04/15/1989</t>
-  </si>
-  <si>
     <t>paigeroberts48</t>
   </si>
   <si>
@@ -929,9 +785,6 @@
     <t>Phillips</t>
   </si>
   <si>
-    <t>07/12/1984</t>
-  </si>
-  <si>
     <t>adamphillips49</t>
   </si>
   <si>
@@ -944,10 +797,157 @@
     <t>Evans</t>
   </si>
   <si>
-    <t>10/24/1999</t>
-  </si>
-  <si>
     <t>emmaevans50</t>
+  </si>
+  <si>
+    <t>01/15/88</t>
+  </si>
+  <si>
+    <t>03/22/92</t>
+  </si>
+  <si>
+    <t>07/08/85</t>
+  </si>
+  <si>
+    <t>11/30/90</t>
+  </si>
+  <si>
+    <t>05/12/87</t>
+  </si>
+  <si>
+    <t>04/18/98</t>
+  </si>
+  <si>
+    <t>09/03/84</t>
+  </si>
+  <si>
+    <t>12/21/93</t>
+  </si>
+  <si>
+    <t>08/10/86</t>
+  </si>
+  <si>
+    <t>02/27/89</t>
+  </si>
+  <si>
+    <t>06/14/83</t>
+  </si>
+  <si>
+    <t>09/09/91</t>
+  </si>
+  <si>
+    <t>01/07/82</t>
+  </si>
+  <si>
+    <t>10/25/88</t>
+  </si>
+  <si>
+    <t>03/17/80</t>
+  </si>
+  <si>
+    <t>07/11/99</t>
+  </si>
+  <si>
+    <t>11/19/87</t>
+  </si>
+  <si>
+    <t>05/22/90</t>
+  </si>
+  <si>
+    <t>04/16/85</t>
+  </si>
+  <si>
+    <t>08/29/94</t>
+  </si>
+  <si>
+    <t>12/13/86</t>
+  </si>
+  <si>
+    <t>06/20/89</t>
+  </si>
+  <si>
+    <t>09/02/92</t>
+  </si>
+  <si>
+    <t>02/08/84</t>
+  </si>
+  <si>
+    <t>04/04/88</t>
+  </si>
+  <si>
+    <t>10/10/99</t>
+  </si>
+  <si>
+    <t>07/27/83</t>
+  </si>
+  <si>
+    <t>01/18/87</t>
+  </si>
+  <si>
+    <t>05/31/81</t>
+  </si>
+  <si>
+    <t>09/14/95</t>
+  </si>
+  <si>
+    <t>03/09/82</t>
+  </si>
+  <si>
+    <t>06/06/88</t>
+  </si>
+  <si>
+    <t>11/22/85</t>
+  </si>
+  <si>
+    <t>08/30/98</t>
+  </si>
+  <si>
+    <t>04/12/84</t>
+  </si>
+  <si>
+    <t>12/01/91</t>
+  </si>
+  <si>
+    <t>07/16/86</t>
+  </si>
+  <si>
+    <t>01/25/93</t>
+  </si>
+  <si>
+    <t>10/05/87</t>
+  </si>
+  <si>
+    <t>03/11/90</t>
+  </si>
+  <si>
+    <t>06/27/94</t>
+  </si>
+  <si>
+    <t>09/17/00</t>
+  </si>
+  <si>
+    <t>02/02/85</t>
+  </si>
+  <si>
+    <t>11/13/88</t>
+  </si>
+  <si>
+    <t>05/21/83</t>
+  </si>
+  <si>
+    <t>08/08/92</t>
+  </si>
+  <si>
+    <t>01/29/86</t>
+  </si>
+  <si>
+    <t>04/15/89</t>
+  </si>
+  <si>
+    <t>07/12/84</t>
+  </si>
+  <si>
+    <t>10/24/99</t>
   </si>
 </sst>
 </file>
@@ -1401,16 +1401,16 @@
         <v>20</v>
       </c>
       <c r="I2" t="s">
+        <v>253</v>
+      </c>
+      <c r="J2" t="s">
         <v>21</v>
-      </c>
-      <c r="J2" t="s">
-        <v>22</v>
       </c>
       <c r="K2">
         <v>2</v>
       </c>
       <c r="L2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="M2" t="b">
         <v>1</v>
@@ -1418,40 +1418,40 @@
     </row>
     <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
         <v>24</v>
       </c>
-      <c r="B3" t="s">
-        <v>14</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>25</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
         <v>26</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F3" t="s">
         <v>27</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G3" t="s">
         <v>28</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>29</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
+        <v>254</v>
+      </c>
+      <c r="J3" t="s">
         <v>30</v>
-      </c>
-      <c r="I3" t="s">
-        <v>31</v>
-      </c>
-      <c r="J3" t="s">
-        <v>32</v>
       </c>
       <c r="K3">
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="M3" t="b">
         <v>1</v>
@@ -1459,19 +1459,19 @@
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B4" t="s">
+        <v>14</v>
+      </c>
+      <c r="C4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D4" t="s">
         <v>34</v>
       </c>
-      <c r="B4" t="s">
-        <v>14</v>
-      </c>
-      <c r="C4" t="s">
+      <c r="E4" t="s">
         <v>35</v>
-      </c>
-      <c r="D4" t="s">
-        <v>36</v>
-      </c>
-      <c r="E4" t="s">
-        <v>37</v>
       </c>
       <c r="F4" t="s">
         <v>18</v>
@@ -1483,16 +1483,16 @@
         <v>20</v>
       </c>
       <c r="I4" t="s">
-        <v>38</v>
+        <v>255</v>
       </c>
       <c r="J4" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K4">
         <v>3</v>
       </c>
       <c r="L4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="M4" t="b">
         <v>1</v>
@@ -1500,40 +1500,40 @@
     </row>
     <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" t="s">
         <v>40</v>
       </c>
-      <c r="B5" t="s">
-        <v>14</v>
-      </c>
-      <c r="C5" t="s">
+      <c r="F5" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" t="s">
         <v>41</v>
       </c>
-      <c r="D5" t="s">
+      <c r="H5" t="s">
         <v>42</v>
       </c>
-      <c r="E5" t="s">
+      <c r="I5" t="s">
+        <v>256</v>
+      </c>
+      <c r="J5" t="s">
+        <v>21</v>
+      </c>
+      <c r="K5">
+        <v>1</v>
+      </c>
+      <c r="L5" t="s">
         <v>43</v>
-      </c>
-      <c r="F5" t="s">
-        <v>28</v>
-      </c>
-      <c r="G5" t="s">
-        <v>44</v>
-      </c>
-      <c r="H5" t="s">
-        <v>45</v>
-      </c>
-      <c r="I5" t="s">
-        <v>46</v>
-      </c>
-      <c r="J5" t="s">
-        <v>22</v>
-      </c>
-      <c r="K5">
-        <v>1</v>
-      </c>
-      <c r="L5" t="s">
-        <v>47</v>
       </c>
       <c r="M5" t="b">
         <v>1</v>
@@ -1541,19 +1541,19 @@
     </row>
     <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="B6" t="s">
         <v>14</v>
       </c>
       <c r="C6" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F6" t="s">
         <v>18</v>
@@ -1565,16 +1565,16 @@
         <v>20</v>
       </c>
       <c r="I6" t="s">
-        <v>52</v>
+        <v>257</v>
       </c>
       <c r="J6" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K6">
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="M6" t="b">
         <v>1</v>
@@ -1582,40 +1582,40 @@
     </row>
     <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
         <v>14</v>
       </c>
       <c r="C7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="D7" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="E7" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F7" t="s">
+        <v>27</v>
+      </c>
+      <c r="G7" t="s">
         <v>28</v>
       </c>
-      <c r="G7" t="s">
-        <v>29</v>
-      </c>
       <c r="H7" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I7" t="s">
-        <v>59</v>
+        <v>258</v>
       </c>
       <c r="J7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="M7" t="b">
         <v>1</v>
@@ -1623,19 +1623,19 @@
     </row>
     <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="B8" t="s">
         <v>14</v>
       </c>
       <c r="C8" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D8" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F8" t="s">
         <v>18</v>
@@ -1647,16 +1647,16 @@
         <v>20</v>
       </c>
       <c r="I8" t="s">
-        <v>65</v>
+        <v>259</v>
       </c>
       <c r="J8" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K8">
         <v>2</v>
       </c>
       <c r="L8" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="M8" t="b">
         <v>1</v>
@@ -1664,40 +1664,40 @@
     </row>
     <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="B9" t="s">
         <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" t="s">
         <v>28</v>
       </c>
-      <c r="G9" t="s">
+      <c r="H9" t="s">
         <v>29</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
+        <v>260</v>
+      </c>
+      <c r="J9" t="s">
         <v>30</v>
-      </c>
-      <c r="I9" t="s">
-        <v>71</v>
-      </c>
-      <c r="J9" t="s">
-        <v>32</v>
       </c>
       <c r="K9">
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="M9" t="b">
         <v>1</v>
@@ -1705,19 +1705,19 @@
     </row>
     <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="B10" t="s">
         <v>14</v>
       </c>
       <c r="C10" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="E10" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F10" t="s">
         <v>18</v>
@@ -1726,19 +1726,19 @@
         <v>19</v>
       </c>
       <c r="H10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I10" t="s">
-        <v>77</v>
+        <v>261</v>
       </c>
       <c r="J10" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K10">
         <v>2</v>
       </c>
       <c r="L10" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="M10" t="b">
         <v>1</v>
@@ -1746,40 +1746,40 @@
     </row>
     <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
         <v>14</v>
       </c>
       <c r="C11" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="D11" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="E11" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="F11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G11" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H11" t="s">
         <v>20</v>
       </c>
       <c r="I11" t="s">
-        <v>83</v>
+        <v>262</v>
       </c>
       <c r="J11" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K11">
         <v>1</v>
       </c>
       <c r="L11" t="s">
-        <v>84</v>
+        <v>74</v>
       </c>
       <c r="M11" t="b">
         <v>1</v>
@@ -1787,19 +1787,19 @@
     </row>
     <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>85</v>
+        <v>75</v>
       </c>
       <c r="B12" t="s">
         <v>14</v>
       </c>
       <c r="C12" t="s">
-        <v>86</v>
+        <v>76</v>
       </c>
       <c r="D12" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="E12" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F12" t="s">
         <v>18</v>
@@ -1811,16 +1811,16 @@
         <v>20</v>
       </c>
       <c r="I12" t="s">
-        <v>89</v>
+        <v>263</v>
       </c>
       <c r="J12" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K12">
         <v>2</v>
       </c>
       <c r="L12" t="s">
-        <v>91</v>
+        <v>80</v>
       </c>
       <c r="M12" t="b">
         <v>1</v>
@@ -1828,40 +1828,40 @@
     </row>
     <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="B13" t="s">
         <v>14</v>
       </c>
       <c r="C13" t="s">
-        <v>93</v>
+        <v>82</v>
       </c>
       <c r="D13" t="s">
-        <v>94</v>
+        <v>83</v>
       </c>
       <c r="E13" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="F13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G13" t="s">
         <v>28</v>
       </c>
-      <c r="G13" t="s">
+      <c r="H13" t="s">
         <v>29</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
+        <v>264</v>
+      </c>
+      <c r="J13" t="s">
         <v>30</v>
-      </c>
-      <c r="I13" t="s">
-        <v>96</v>
-      </c>
-      <c r="J13" t="s">
-        <v>32</v>
       </c>
       <c r="K13">
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>97</v>
+        <v>85</v>
       </c>
       <c r="M13" t="b">
         <v>1</v>
@@ -1869,19 +1869,19 @@
     </row>
     <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>98</v>
+        <v>86</v>
       </c>
       <c r="B14" t="s">
         <v>14</v>
       </c>
       <c r="C14" t="s">
-        <v>99</v>
+        <v>87</v>
       </c>
       <c r="D14" t="s">
-        <v>100</v>
+        <v>88</v>
       </c>
       <c r="E14" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F14" t="s">
         <v>18</v>
@@ -1893,16 +1893,16 @@
         <v>20</v>
       </c>
       <c r="I14" t="s">
-        <v>102</v>
+        <v>265</v>
       </c>
       <c r="J14" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K14">
         <v>3</v>
       </c>
       <c r="L14" t="s">
-        <v>103</v>
+        <v>90</v>
       </c>
       <c r="M14" t="b">
         <v>1</v>
@@ -1910,40 +1910,40 @@
     </row>
     <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>104</v>
+        <v>91</v>
       </c>
       <c r="B15" t="s">
         <v>14</v>
       </c>
       <c r="C15" t="s">
-        <v>105</v>
+        <v>92</v>
       </c>
       <c r="D15" t="s">
-        <v>106</v>
+        <v>93</v>
       </c>
       <c r="E15" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="F15" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G15" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H15" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I15" t="s">
-        <v>108</v>
+        <v>266</v>
       </c>
       <c r="J15" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K15">
         <v>1</v>
       </c>
       <c r="L15" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="M15" t="b">
         <v>1</v>
@@ -1951,40 +1951,40 @@
     </row>
     <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="B16" t="s">
         <v>14</v>
       </c>
       <c r="C16" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="D16" t="s">
-        <v>112</v>
+        <v>98</v>
       </c>
       <c r="E16" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="F16" t="s">
         <v>18</v>
       </c>
       <c r="G16" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="H16" t="s">
         <v>20</v>
       </c>
       <c r="I16" t="s">
-        <v>115</v>
+        <v>267</v>
       </c>
       <c r="J16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K16">
         <v>2</v>
       </c>
       <c r="L16" t="s">
-        <v>116</v>
+        <v>101</v>
       </c>
       <c r="M16" t="b">
         <v>1</v>
@@ -1992,40 +1992,40 @@
     </row>
     <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>117</v>
+        <v>102</v>
       </c>
       <c r="B17" t="s">
         <v>14</v>
       </c>
       <c r="C17" t="s">
-        <v>118</v>
+        <v>103</v>
       </c>
       <c r="D17" t="s">
-        <v>119</v>
+        <v>104</v>
       </c>
       <c r="E17" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="F17" t="s">
+        <v>27</v>
+      </c>
+      <c r="G17" t="s">
         <v>28</v>
       </c>
-      <c r="G17" t="s">
-        <v>29</v>
-      </c>
       <c r="H17" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I17" t="s">
-        <v>121</v>
+        <v>268</v>
       </c>
       <c r="J17" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K17">
         <v>0</v>
       </c>
       <c r="L17" t="s">
-        <v>122</v>
+        <v>106</v>
       </c>
       <c r="M17" t="b">
         <v>1</v>
@@ -2033,19 +2033,19 @@
     </row>
     <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>123</v>
+        <v>107</v>
       </c>
       <c r="B18" t="s">
         <v>14</v>
       </c>
       <c r="C18" t="s">
-        <v>124</v>
+        <v>108</v>
       </c>
       <c r="D18" t="s">
-        <v>125</v>
+        <v>109</v>
       </c>
       <c r="E18" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="F18" t="s">
         <v>18</v>
@@ -2057,16 +2057,16 @@
         <v>20</v>
       </c>
       <c r="I18" t="s">
-        <v>127</v>
+        <v>269</v>
       </c>
       <c r="J18" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K18">
         <v>2</v>
       </c>
       <c r="L18" t="s">
-        <v>128</v>
+        <v>111</v>
       </c>
       <c r="M18" t="b">
         <v>1</v>
@@ -2074,40 +2074,40 @@
     </row>
     <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>129</v>
+        <v>112</v>
       </c>
       <c r="B19" t="s">
         <v>14</v>
       </c>
       <c r="C19" t="s">
-        <v>130</v>
+        <v>113</v>
       </c>
       <c r="D19" t="s">
-        <v>131</v>
+        <v>114</v>
       </c>
       <c r="E19" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="F19" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G19" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H19" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I19" t="s">
-        <v>133</v>
+        <v>270</v>
       </c>
       <c r="J19" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K19">
         <v>1</v>
       </c>
       <c r="L19" t="s">
-        <v>134</v>
+        <v>116</v>
       </c>
       <c r="M19" t="b">
         <v>1</v>
@@ -2115,19 +2115,19 @@
     </row>
     <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="B20" t="s">
         <v>14</v>
       </c>
       <c r="C20" t="s">
-        <v>136</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
-        <v>137</v>
+        <v>119</v>
       </c>
       <c r="E20" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="F20" t="s">
         <v>18</v>
@@ -2136,19 +2136,19 @@
         <v>19</v>
       </c>
       <c r="H20" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I20" t="s">
-        <v>139</v>
+        <v>271</v>
       </c>
       <c r="J20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K20">
         <v>0</v>
       </c>
       <c r="L20" t="s">
-        <v>140</v>
+        <v>121</v>
       </c>
       <c r="M20" t="b">
         <v>1</v>
@@ -2156,40 +2156,40 @@
     </row>
     <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>141</v>
+        <v>122</v>
       </c>
       <c r="B21" t="s">
         <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>142</v>
+        <v>123</v>
       </c>
       <c r="D21" t="s">
-        <v>143</v>
+        <v>124</v>
       </c>
       <c r="E21" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F21" t="s">
+        <v>27</v>
+      </c>
+      <c r="G21" t="s">
         <v>28</v>
-      </c>
-      <c r="G21" t="s">
-        <v>29</v>
       </c>
       <c r="H21" t="s">
         <v>20</v>
       </c>
       <c r="I21" t="s">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="J21" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K21">
         <v>0</v>
       </c>
       <c r="L21" t="s">
-        <v>146</v>
+        <v>126</v>
       </c>
       <c r="M21" t="b">
         <v>1</v>
@@ -2197,19 +2197,19 @@
     </row>
     <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>147</v>
+        <v>127</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
       </c>
       <c r="C22" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="D22" t="s">
-        <v>149</v>
+        <v>129</v>
       </c>
       <c r="E22" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="F22" t="s">
         <v>18</v>
@@ -2221,16 +2221,16 @@
         <v>20</v>
       </c>
       <c r="I22" t="s">
-        <v>151</v>
+        <v>273</v>
       </c>
       <c r="J22" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K22">
         <v>2</v>
       </c>
       <c r="L22" t="s">
-        <v>152</v>
+        <v>131</v>
       </c>
       <c r="M22" t="b">
         <v>1</v>
@@ -2238,40 +2238,40 @@
     </row>
     <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>153</v>
+        <v>132</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
       </c>
       <c r="C23" t="s">
-        <v>154</v>
+        <v>133</v>
       </c>
       <c r="D23" t="s">
-        <v>155</v>
+        <v>134</v>
       </c>
       <c r="E23" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="F23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G23" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H23" t="s">
         <v>20</v>
       </c>
       <c r="I23" t="s">
-        <v>157</v>
+        <v>274</v>
       </c>
       <c r="J23" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K23">
         <v>2</v>
       </c>
       <c r="L23" t="s">
-        <v>158</v>
+        <v>136</v>
       </c>
       <c r="M23" t="b">
         <v>1</v>
@@ -2279,19 +2279,19 @@
     </row>
     <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>159</v>
+        <v>137</v>
       </c>
       <c r="B24" t="s">
         <v>14</v>
       </c>
       <c r="C24" t="s">
-        <v>160</v>
+        <v>138</v>
       </c>
       <c r="D24" t="s">
-        <v>161</v>
+        <v>139</v>
       </c>
       <c r="E24" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="F24" t="s">
         <v>18</v>
@@ -2300,19 +2300,19 @@
         <v>19</v>
       </c>
       <c r="H24" t="s">
+        <v>29</v>
+      </c>
+      <c r="I24" t="s">
+        <v>275</v>
+      </c>
+      <c r="J24" t="s">
         <v>30</v>
-      </c>
-      <c r="I24" t="s">
-        <v>163</v>
-      </c>
-      <c r="J24" t="s">
-        <v>32</v>
       </c>
       <c r="K24">
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>164</v>
+        <v>141</v>
       </c>
       <c r="M24" t="b">
         <v>1</v>
@@ -2320,40 +2320,40 @@
     </row>
     <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>165</v>
+        <v>142</v>
       </c>
       <c r="B25" t="s">
         <v>14</v>
       </c>
       <c r="C25" t="s">
-        <v>166</v>
+        <v>143</v>
       </c>
       <c r="D25" t="s">
-        <v>167</v>
+        <v>144</v>
       </c>
       <c r="E25" t="s">
-        <v>168</v>
+        <v>145</v>
       </c>
       <c r="F25" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G25" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="H25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I25" t="s">
-        <v>169</v>
+        <v>276</v>
       </c>
       <c r="J25" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K25">
         <v>1</v>
       </c>
       <c r="L25" t="s">
-        <v>170</v>
+        <v>146</v>
       </c>
       <c r="M25" t="b">
         <v>1</v>
@@ -2361,19 +2361,19 @@
     </row>
     <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>171</v>
+        <v>147</v>
       </c>
       <c r="B26" t="s">
         <v>14</v>
       </c>
       <c r="C26" t="s">
-        <v>172</v>
+        <v>148</v>
       </c>
       <c r="D26" t="s">
-        <v>173</v>
+        <v>149</v>
       </c>
       <c r="E26" t="s">
-        <v>174</v>
+        <v>150</v>
       </c>
       <c r="F26" t="s">
         <v>18</v>
@@ -2385,16 +2385,16 @@
         <v>20</v>
       </c>
       <c r="I26" t="s">
-        <v>175</v>
+        <v>277</v>
       </c>
       <c r="J26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K26">
         <v>2</v>
       </c>
       <c r="L26" t="s">
-        <v>176</v>
+        <v>151</v>
       </c>
       <c r="M26" t="b">
         <v>1</v>
@@ -2402,40 +2402,40 @@
     </row>
     <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>177</v>
+        <v>152</v>
       </c>
       <c r="B27" t="s">
         <v>14</v>
       </c>
       <c r="C27" t="s">
-        <v>178</v>
+        <v>153</v>
       </c>
       <c r="D27" t="s">
-        <v>179</v>
+        <v>154</v>
       </c>
       <c r="E27" t="s">
-        <v>180</v>
+        <v>155</v>
       </c>
       <c r="F27" t="s">
+        <v>27</v>
+      </c>
+      <c r="G27" t="s">
         <v>28</v>
       </c>
-      <c r="G27" t="s">
-        <v>29</v>
-      </c>
       <c r="H27" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I27" t="s">
-        <v>181</v>
+        <v>278</v>
       </c>
       <c r="J27" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K27">
         <v>0</v>
       </c>
       <c r="L27" t="s">
-        <v>182</v>
+        <v>156</v>
       </c>
       <c r="M27" t="b">
         <v>1</v>
@@ -2443,16 +2443,16 @@
     </row>
     <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>183</v>
+        <v>157</v>
       </c>
       <c r="B28" t="s">
         <v>14</v>
       </c>
       <c r="C28" t="s">
-        <v>184</v>
+        <v>158</v>
       </c>
       <c r="D28" t="s">
-        <v>185</v>
+        <v>159</v>
       </c>
       <c r="E28" t="s">
         <v>17</v>
@@ -2467,16 +2467,16 @@
         <v>20</v>
       </c>
       <c r="I28" t="s">
-        <v>186</v>
+        <v>279</v>
       </c>
       <c r="J28" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K28">
         <v>3</v>
       </c>
       <c r="L28" t="s">
-        <v>187</v>
+        <v>160</v>
       </c>
       <c r="M28" t="b">
         <v>1</v>
@@ -2484,40 +2484,40 @@
     </row>
     <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>188</v>
+        <v>161</v>
       </c>
       <c r="B29" t="s">
         <v>14</v>
       </c>
       <c r="C29" t="s">
-        <v>189</v>
+        <v>162</v>
       </c>
       <c r="D29" t="s">
-        <v>190</v>
+        <v>163</v>
       </c>
       <c r="E29" t="s">
+        <v>26</v>
+      </c>
+      <c r="F29" t="s">
         <v>27</v>
       </c>
-      <c r="F29" t="s">
-        <v>28</v>
-      </c>
       <c r="G29" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H29" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I29" t="s">
-        <v>191</v>
+        <v>280</v>
       </c>
       <c r="J29" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K29">
         <v>1</v>
       </c>
       <c r="L29" t="s">
-        <v>192</v>
+        <v>164</v>
       </c>
       <c r="M29" t="b">
         <v>1</v>
@@ -2525,19 +2525,19 @@
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>193</v>
+        <v>165</v>
       </c>
       <c r="B30" t="s">
         <v>14</v>
       </c>
       <c r="C30" t="s">
-        <v>194</v>
+        <v>166</v>
       </c>
       <c r="D30" t="s">
-        <v>195</v>
+        <v>167</v>
       </c>
       <c r="E30" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="F30" t="s">
         <v>18</v>
@@ -2549,16 +2549,16 @@
         <v>20</v>
       </c>
       <c r="I30" t="s">
-        <v>196</v>
+        <v>281</v>
       </c>
       <c r="J30" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K30">
         <v>2</v>
       </c>
       <c r="L30" t="s">
-        <v>197</v>
+        <v>168</v>
       </c>
       <c r="M30" t="b">
         <v>1</v>
@@ -2566,40 +2566,40 @@
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>198</v>
+        <v>169</v>
       </c>
       <c r="B31" t="s">
         <v>14</v>
       </c>
       <c r="C31" t="s">
-        <v>199</v>
+        <v>170</v>
       </c>
       <c r="D31" t="s">
-        <v>200</v>
+        <v>171</v>
       </c>
       <c r="E31" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="F31" t="s">
+        <v>27</v>
+      </c>
+      <c r="G31" t="s">
         <v>28</v>
       </c>
-      <c r="G31" t="s">
+      <c r="H31" t="s">
         <v>29</v>
       </c>
-      <c r="H31" t="s">
+      <c r="I31" t="s">
+        <v>282</v>
+      </c>
+      <c r="J31" t="s">
         <v>30</v>
-      </c>
-      <c r="I31" t="s">
-        <v>201</v>
-      </c>
-      <c r="J31" t="s">
-        <v>32</v>
       </c>
       <c r="K31">
         <v>0</v>
       </c>
       <c r="L31" t="s">
-        <v>202</v>
+        <v>172</v>
       </c>
       <c r="M31" t="b">
         <v>1</v>
@@ -2607,19 +2607,19 @@
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>203</v>
+        <v>173</v>
       </c>
       <c r="B32" t="s">
         <v>14</v>
       </c>
       <c r="C32" t="s">
-        <v>204</v>
+        <v>174</v>
       </c>
       <c r="D32" t="s">
-        <v>205</v>
+        <v>175</v>
       </c>
       <c r="E32" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="F32" t="s">
         <v>18</v>
@@ -2631,16 +2631,16 @@
         <v>20</v>
       </c>
       <c r="I32" t="s">
-        <v>206</v>
+        <v>283</v>
       </c>
       <c r="J32" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K32">
         <v>2</v>
       </c>
       <c r="L32" t="s">
-        <v>207</v>
+        <v>176</v>
       </c>
       <c r="M32" t="b">
         <v>1</v>
@@ -2648,40 +2648,40 @@
     </row>
     <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>208</v>
+        <v>177</v>
       </c>
       <c r="B33" t="s">
         <v>14</v>
       </c>
       <c r="C33" t="s">
-        <v>209</v>
+        <v>178</v>
       </c>
       <c r="D33" t="s">
-        <v>210</v>
+        <v>179</v>
       </c>
       <c r="E33" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="F33" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G33" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H33" t="s">
         <v>20</v>
       </c>
       <c r="I33" t="s">
-        <v>211</v>
+        <v>284</v>
       </c>
       <c r="J33" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K33">
         <v>2</v>
       </c>
       <c r="L33" t="s">
-        <v>212</v>
+        <v>180</v>
       </c>
       <c r="M33" t="b">
         <v>1</v>
@@ -2689,40 +2689,40 @@
     </row>
     <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>213</v>
+        <v>181</v>
       </c>
       <c r="B34" t="s">
         <v>14</v>
       </c>
       <c r="C34" t="s">
-        <v>214</v>
+        <v>182</v>
       </c>
       <c r="D34" t="s">
-        <v>215</v>
+        <v>183</v>
       </c>
       <c r="E34" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="F34" t="s">
         <v>18</v>
       </c>
       <c r="G34" t="s">
-        <v>114</v>
+        <v>100</v>
       </c>
       <c r="H34" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I34" t="s">
-        <v>216</v>
+        <v>285</v>
       </c>
       <c r="J34" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K34">
         <v>1</v>
       </c>
       <c r="L34" t="s">
-        <v>217</v>
+        <v>184</v>
       </c>
       <c r="M34" t="b">
         <v>1</v>
@@ -2730,40 +2730,40 @@
     </row>
     <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>218</v>
+        <v>185</v>
       </c>
       <c r="B35" t="s">
         <v>14</v>
       </c>
       <c r="C35" t="s">
-        <v>219</v>
+        <v>186</v>
       </c>
       <c r="D35" t="s">
-        <v>220</v>
+        <v>187</v>
       </c>
       <c r="E35" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="F35" t="s">
+        <v>27</v>
+      </c>
+      <c r="G35" t="s">
         <v>28</v>
       </c>
-      <c r="G35" t="s">
-        <v>29</v>
-      </c>
       <c r="H35" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I35" t="s">
-        <v>221</v>
+        <v>286</v>
       </c>
       <c r="J35" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K35">
         <v>0</v>
       </c>
       <c r="L35" t="s">
-        <v>222</v>
+        <v>188</v>
       </c>
       <c r="M35" t="b">
         <v>1</v>
@@ -2771,19 +2771,19 @@
     </row>
     <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>223</v>
+        <v>189</v>
       </c>
       <c r="B36" t="s">
         <v>14</v>
       </c>
       <c r="C36" t="s">
-        <v>224</v>
+        <v>190</v>
       </c>
       <c r="D36" t="s">
-        <v>225</v>
+        <v>191</v>
       </c>
       <c r="E36" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="F36" t="s">
         <v>18</v>
@@ -2795,16 +2795,16 @@
         <v>20</v>
       </c>
       <c r="I36" t="s">
-        <v>226</v>
+        <v>287</v>
       </c>
       <c r="J36" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K36">
         <v>3</v>
       </c>
       <c r="L36" t="s">
-        <v>227</v>
+        <v>192</v>
       </c>
       <c r="M36" t="b">
         <v>1</v>
@@ -2812,40 +2812,40 @@
     </row>
     <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>228</v>
+        <v>193</v>
       </c>
       <c r="B37" t="s">
         <v>14</v>
       </c>
       <c r="C37" t="s">
-        <v>229</v>
+        <v>194</v>
       </c>
       <c r="D37" t="s">
-        <v>230</v>
+        <v>195</v>
       </c>
       <c r="E37" t="s">
-        <v>82</v>
+        <v>73</v>
       </c>
       <c r="F37" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G37" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H37" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="I37" t="s">
-        <v>231</v>
+        <v>288</v>
       </c>
       <c r="J37" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K37">
         <v>1</v>
       </c>
       <c r="L37" t="s">
-        <v>232</v>
+        <v>196</v>
       </c>
       <c r="M37" t="b">
         <v>1</v>
@@ -2853,19 +2853,19 @@
     </row>
     <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>233</v>
+        <v>197</v>
       </c>
       <c r="B38" t="s">
         <v>14</v>
       </c>
       <c r="C38" t="s">
-        <v>234</v>
+        <v>198</v>
       </c>
       <c r="D38" t="s">
-        <v>235</v>
+        <v>199</v>
       </c>
       <c r="E38" t="s">
-        <v>88</v>
+        <v>78</v>
       </c>
       <c r="F38" t="s">
         <v>18</v>
@@ -2877,16 +2877,16 @@
         <v>20</v>
       </c>
       <c r="I38" t="s">
-        <v>236</v>
+        <v>289</v>
       </c>
       <c r="J38" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K38">
         <v>0</v>
       </c>
       <c r="L38" t="s">
-        <v>237</v>
+        <v>200</v>
       </c>
       <c r="M38" t="b">
         <v>1</v>
@@ -2894,40 +2894,40 @@
     </row>
     <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>238</v>
+        <v>201</v>
       </c>
       <c r="B39" t="s">
         <v>14</v>
       </c>
       <c r="C39" t="s">
-        <v>239</v>
+        <v>202</v>
       </c>
       <c r="D39" t="s">
-        <v>240</v>
+        <v>203</v>
       </c>
       <c r="E39" t="s">
-        <v>95</v>
+        <v>84</v>
       </c>
       <c r="F39" t="s">
+        <v>27</v>
+      </c>
+      <c r="G39" t="s">
         <v>28</v>
       </c>
-      <c r="G39" t="s">
-        <v>29</v>
-      </c>
       <c r="H39" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I39" t="s">
-        <v>241</v>
+        <v>290</v>
       </c>
       <c r="J39" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K39">
         <v>0</v>
       </c>
       <c r="L39" t="s">
-        <v>242</v>
+        <v>204</v>
       </c>
       <c r="M39" t="b">
         <v>1</v>
@@ -2935,19 +2935,19 @@
     </row>
     <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>243</v>
+        <v>205</v>
       </c>
       <c r="B40" t="s">
         <v>14</v>
       </c>
       <c r="C40" t="s">
-        <v>244</v>
+        <v>206</v>
       </c>
       <c r="D40" t="s">
-        <v>245</v>
+        <v>207</v>
       </c>
       <c r="E40" t="s">
-        <v>101</v>
+        <v>89</v>
       </c>
       <c r="F40" t="s">
         <v>18</v>
@@ -2959,16 +2959,16 @@
         <v>20</v>
       </c>
       <c r="I40" t="s">
-        <v>246</v>
+        <v>291</v>
       </c>
       <c r="J40" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K40">
         <v>2</v>
       </c>
       <c r="L40" t="s">
-        <v>247</v>
+        <v>208</v>
       </c>
       <c r="M40" t="b">
         <v>1</v>
@@ -2976,40 +2976,40 @@
     </row>
     <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>248</v>
+        <v>209</v>
       </c>
       <c r="B41" t="s">
         <v>14</v>
       </c>
       <c r="C41" t="s">
-        <v>249</v>
+        <v>210</v>
       </c>
       <c r="D41" t="s">
-        <v>250</v>
+        <v>211</v>
       </c>
       <c r="E41" t="s">
-        <v>107</v>
+        <v>94</v>
       </c>
       <c r="F41" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G41" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H41" t="s">
         <v>20</v>
       </c>
       <c r="I41" t="s">
-        <v>251</v>
+        <v>292</v>
       </c>
       <c r="J41" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K41">
         <v>1</v>
       </c>
       <c r="L41" t="s">
-        <v>252</v>
+        <v>212</v>
       </c>
       <c r="M41" t="b">
         <v>1</v>
@@ -3017,19 +3017,19 @@
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>253</v>
+        <v>213</v>
       </c>
       <c r="B42" t="s">
         <v>14</v>
       </c>
       <c r="C42" t="s">
-        <v>254</v>
+        <v>214</v>
       </c>
       <c r="D42" t="s">
-        <v>255</v>
+        <v>215</v>
       </c>
       <c r="E42" t="s">
-        <v>113</v>
+        <v>99</v>
       </c>
       <c r="F42" t="s">
         <v>18</v>
@@ -3038,19 +3038,19 @@
         <v>19</v>
       </c>
       <c r="H42" t="s">
+        <v>29</v>
+      </c>
+      <c r="I42" t="s">
+        <v>293</v>
+      </c>
+      <c r="J42" t="s">
         <v>30</v>
-      </c>
-      <c r="I42" t="s">
-        <v>256</v>
-      </c>
-      <c r="J42" t="s">
-        <v>32</v>
       </c>
       <c r="K42">
         <v>0</v>
       </c>
       <c r="L42" t="s">
-        <v>257</v>
+        <v>216</v>
       </c>
       <c r="M42" t="b">
         <v>1</v>
@@ -3058,40 +3058,40 @@
     </row>
     <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>258</v>
+        <v>217</v>
       </c>
       <c r="B43" t="s">
         <v>14</v>
       </c>
       <c r="C43" t="s">
-        <v>259</v>
+        <v>218</v>
       </c>
       <c r="D43" t="s">
-        <v>260</v>
+        <v>219</v>
       </c>
       <c r="E43" t="s">
-        <v>120</v>
+        <v>105</v>
       </c>
       <c r="F43" t="s">
+        <v>27</v>
+      </c>
+      <c r="G43" t="s">
         <v>28</v>
       </c>
-      <c r="G43" t="s">
-        <v>29</v>
-      </c>
       <c r="H43" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I43" t="s">
-        <v>261</v>
+        <v>294</v>
       </c>
       <c r="J43" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K43">
         <v>0</v>
       </c>
       <c r="L43" t="s">
-        <v>262</v>
+        <v>220</v>
       </c>
       <c r="M43" t="b">
         <v>1</v>
@@ -3099,19 +3099,19 @@
     </row>
     <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>263</v>
+        <v>221</v>
       </c>
       <c r="B44" t="s">
         <v>14</v>
       </c>
       <c r="C44" t="s">
-        <v>264</v>
+        <v>222</v>
       </c>
       <c r="D44" t="s">
-        <v>265</v>
+        <v>223</v>
       </c>
       <c r="E44" t="s">
-        <v>126</v>
+        <v>110</v>
       </c>
       <c r="F44" t="s">
         <v>18</v>
@@ -3123,16 +3123,16 @@
         <v>20</v>
       </c>
       <c r="I44" t="s">
-        <v>266</v>
+        <v>295</v>
       </c>
       <c r="J44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K44">
         <v>2</v>
       </c>
       <c r="L44" t="s">
-        <v>267</v>
+        <v>224</v>
       </c>
       <c r="M44" t="b">
         <v>1</v>
@@ -3140,40 +3140,40 @@
     </row>
     <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>268</v>
+        <v>225</v>
       </c>
       <c r="B45" t="s">
         <v>14</v>
       </c>
       <c r="C45" t="s">
-        <v>269</v>
+        <v>226</v>
       </c>
       <c r="D45" t="s">
-        <v>270</v>
+        <v>227</v>
       </c>
       <c r="E45" t="s">
-        <v>132</v>
+        <v>115</v>
       </c>
       <c r="F45" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G45" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H45" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I45" t="s">
-        <v>271</v>
+        <v>296</v>
       </c>
       <c r="J45" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K45">
         <v>1</v>
       </c>
       <c r="L45" t="s">
-        <v>272</v>
+        <v>228</v>
       </c>
       <c r="M45" t="b">
         <v>1</v>
@@ -3181,19 +3181,19 @@
     </row>
     <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>273</v>
+        <v>229</v>
       </c>
       <c r="B46" t="s">
         <v>14</v>
       </c>
       <c r="C46" t="s">
-        <v>274</v>
+        <v>230</v>
       </c>
       <c r="D46" t="s">
-        <v>275</v>
+        <v>231</v>
       </c>
       <c r="E46" t="s">
-        <v>138</v>
+        <v>120</v>
       </c>
       <c r="F46" t="s">
         <v>18</v>
@@ -3205,16 +3205,16 @@
         <v>20</v>
       </c>
       <c r="I46" t="s">
-        <v>276</v>
+        <v>297</v>
       </c>
       <c r="J46" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K46">
         <v>3</v>
       </c>
       <c r="L46" t="s">
-        <v>277</v>
+        <v>232</v>
       </c>
       <c r="M46" t="b">
         <v>1</v>
@@ -3222,40 +3222,40 @@
     </row>
     <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>278</v>
+        <v>233</v>
       </c>
       <c r="B47" t="s">
         <v>14</v>
       </c>
       <c r="C47" t="s">
-        <v>279</v>
+        <v>234</v>
       </c>
       <c r="D47" t="s">
-        <v>280</v>
+        <v>235</v>
       </c>
       <c r="E47" t="s">
-        <v>144</v>
+        <v>125</v>
       </c>
       <c r="F47" t="s">
+        <v>27</v>
+      </c>
+      <c r="G47" t="s">
         <v>28</v>
       </c>
-      <c r="G47" t="s">
+      <c r="H47" t="s">
         <v>29</v>
       </c>
-      <c r="H47" t="s">
+      <c r="I47" t="s">
+        <v>298</v>
+      </c>
+      <c r="J47" t="s">
         <v>30</v>
-      </c>
-      <c r="I47" t="s">
-        <v>281</v>
-      </c>
-      <c r="J47" t="s">
-        <v>32</v>
       </c>
       <c r="K47">
         <v>0</v>
       </c>
       <c r="L47" t="s">
-        <v>282</v>
+        <v>236</v>
       </c>
       <c r="M47" t="b">
         <v>1</v>
@@ -3263,19 +3263,19 @@
     </row>
     <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>283</v>
+        <v>237</v>
       </c>
       <c r="B48" t="s">
         <v>14</v>
       </c>
       <c r="C48" t="s">
-        <v>284</v>
+        <v>238</v>
       </c>
       <c r="D48" t="s">
-        <v>285</v>
+        <v>239</v>
       </c>
       <c r="E48" t="s">
-        <v>150</v>
+        <v>130</v>
       </c>
       <c r="F48" t="s">
         <v>18</v>
@@ -3287,16 +3287,16 @@
         <v>20</v>
       </c>
       <c r="I48" t="s">
-        <v>286</v>
+        <v>299</v>
       </c>
       <c r="J48" t="s">
-        <v>90</v>
+        <v>79</v>
       </c>
       <c r="K48">
         <v>1</v>
       </c>
       <c r="L48" t="s">
-        <v>287</v>
+        <v>240</v>
       </c>
       <c r="M48" t="b">
         <v>1</v>
@@ -3304,40 +3304,40 @@
     </row>
     <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>288</v>
+        <v>241</v>
       </c>
       <c r="B49" t="s">
         <v>14</v>
       </c>
       <c r="C49" t="s">
-        <v>289</v>
+        <v>242</v>
       </c>
       <c r="D49" t="s">
-        <v>290</v>
+        <v>243</v>
       </c>
       <c r="E49" t="s">
-        <v>156</v>
+        <v>135</v>
       </c>
       <c r="F49" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G49" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="H49" t="s">
         <v>20</v>
       </c>
       <c r="I49" t="s">
-        <v>291</v>
+        <v>300</v>
       </c>
       <c r="J49" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K49">
         <v>2</v>
       </c>
       <c r="L49" t="s">
-        <v>292</v>
+        <v>244</v>
       </c>
       <c r="M49" t="b">
         <v>1</v>
@@ -3345,19 +3345,19 @@
     </row>
     <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>293</v>
+        <v>245</v>
       </c>
       <c r="B50" t="s">
         <v>14</v>
       </c>
       <c r="C50" t="s">
-        <v>294</v>
+        <v>246</v>
       </c>
       <c r="D50" t="s">
-        <v>295</v>
+        <v>247</v>
       </c>
       <c r="E50" t="s">
-        <v>162</v>
+        <v>140</v>
       </c>
       <c r="F50" t="s">
         <v>18</v>
@@ -3366,19 +3366,19 @@
         <v>19</v>
       </c>
       <c r="H50" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I50" t="s">
-        <v>296</v>
+        <v>301</v>
       </c>
       <c r="J50" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="K50">
         <v>2</v>
       </c>
       <c r="L50" t="s">
-        <v>297</v>
+        <v>248</v>
       </c>
       <c r="M50" t="b">
         <v>1</v>
@@ -3386,40 +3386,40 @@
     </row>
     <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>298</v>
+        <v>249</v>
       </c>
       <c r="B51" t="s">
         <v>14</v>
       </c>
       <c r="C51" t="s">
-        <v>299</v>
+        <v>250</v>
       </c>
       <c r="D51" t="s">
-        <v>300</v>
+        <v>251</v>
       </c>
       <c r="E51" t="s">
-        <v>168</v>
+        <v>145</v>
       </c>
       <c r="F51" t="s">
+        <v>27</v>
+      </c>
+      <c r="G51" t="s">
         <v>28</v>
       </c>
-      <c r="G51" t="s">
-        <v>29</v>
-      </c>
       <c r="H51" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="I51" t="s">
-        <v>301</v>
+        <v>302</v>
       </c>
       <c r="J51" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="K51">
         <v>0</v>
       </c>
       <c r="L51" t="s">
-        <v>302</v>
+        <v>252</v>
       </c>
       <c r="M51" t="b">
         <v>1</v>

</xml_diff>